<commit_message>
Ajout de la mise en forme dans le excel, il manque plus qu'a bouger la justification et voir pour la taille des cases
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t xml:space="preserve">Matrice NOM DU PROJET</t>
   </si>
@@ -71,49 +71,7 @@
     <t xml:space="preserve">Justification Infodip </t>
   </si>
   <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pourquoi avoir choisi ce composant ? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audio component</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Network</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Out of band management</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Storage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Warranty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">License</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other</t>
   </si>
   <si>
     <t xml:space="preserve">Pourquoi avoir avoir choisi ce produit ? </t>
@@ -369,127 +327,127 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -849,31 +807,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:H51"/>
+  <dimension ref="B2:H51"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="37.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="42.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="37.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="18.29"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2"/>
       <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3" t="s">
@@ -951,55 +901,42 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="19" t="s">
-        <v>16</v>
-      </c>
+      <c r="B13" s="19"/>
       <c r="C13" s="20"/>
       <c r="D13" s="21"/>
       <c r="E13" s="22"/>
       <c r="F13" s="21"/>
       <c r="G13" s="23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="19" t="s">
-        <v>18</v>
-      </c>
+      <c r="B14" s="19"/>
       <c r="C14" s="25"/>
       <c r="D14" s="22"/>
       <c r="E14" s="22"/>
       <c r="F14" s="22"/>
       <c r="G14" s="23"/>
-      <c r="H14" s="1"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="19" t="s">
-        <v>19</v>
-      </c>
+      <c r="B15" s="19"/>
       <c r="C15" s="25"/>
       <c r="D15" s="22"/>
       <c r="E15" s="22"/>
       <c r="F15" s="22"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="1"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="19" t="s">
-        <v>20</v>
-      </c>
+      <c r="B16" s="19"/>
       <c r="C16" s="25"/>
       <c r="D16" s="22"/>
       <c r="E16" s="22"/>
       <c r="F16" s="22"/>
       <c r="G16" s="23"/>
-      <c r="H16" s="1"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="B17" s="19"/>
       <c r="C17" s="25"/>
       <c r="D17" s="22"/>
       <c r="E17" s="22"/>
@@ -1008,9 +945,7 @@
       <c r="H17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="19" t="s">
-        <v>22</v>
-      </c>
+      <c r="B18" s="19"/>
       <c r="C18" s="25"/>
       <c r="D18" s="22"/>
       <c r="E18" s="22"/>
@@ -1019,42 +954,31 @@
       <c r="H18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="19" t="s">
-        <v>23</v>
-      </c>
+      <c r="B19" s="19"/>
       <c r="C19" s="25"/>
       <c r="D19" s="22"/>
       <c r="E19" s="22"/>
       <c r="F19" s="22"/>
       <c r="G19" s="23"/>
-      <c r="H19" s="1"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="19" t="s">
-        <v>24</v>
-      </c>
+      <c r="B20" s="19"/>
       <c r="C20" s="25"/>
       <c r="D20" s="22"/>
       <c r="E20" s="22"/>
       <c r="F20" s="22"/>
       <c r="G20" s="23"/>
-      <c r="H20" s="1"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="19" t="s">
-        <v>25</v>
-      </c>
+      <c r="B21" s="19"/>
       <c r="C21" s="25"/>
       <c r="D21" s="22"/>
       <c r="E21" s="22"/>
       <c r="F21" s="22"/>
       <c r="G21" s="23"/>
-      <c r="H21" s="1"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="19" t="s">
-        <v>26</v>
-      </c>
+      <c r="B22" s="19"/>
       <c r="C22" s="25"/>
       <c r="D22" s="22"/>
       <c r="E22" s="22"/>
@@ -1063,9 +987,7 @@
       <c r="H22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="19" t="s">
-        <v>27</v>
-      </c>
+      <c r="B23" s="19"/>
       <c r="C23" s="25"/>
       <c r="D23" s="22"/>
       <c r="E23" s="22"/>
@@ -1074,20 +996,15 @@
       <c r="H23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="19" t="s">
-        <v>28</v>
-      </c>
+      <c r="B24" s="19"/>
       <c r="C24" s="25"/>
       <c r="D24" s="22"/>
       <c r="E24" s="22"/>
       <c r="F24" s="22"/>
       <c r="G24" s="23"/>
-      <c r="H24" s="1"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="19" t="s">
-        <v>29</v>
-      </c>
+      <c r="B25" s="19"/>
       <c r="C25" s="25"/>
       <c r="D25" s="22"/>
       <c r="E25" s="22"/>
@@ -1096,9 +1013,7 @@
       <c r="H25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="19" t="s">
-        <v>30</v>
-      </c>
+      <c r="B26" s="19"/>
       <c r="C26" s="25"/>
       <c r="D26" s="22"/>
       <c r="E26" s="22"/>
@@ -1111,7 +1026,7 @@
         <v>15</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1132,7 +1047,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{2AF79554-2E10-4247-989F-62799AAC8AC7}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{B0658272-EA1E-46B9-B6CA-45705880BE4A}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1142,7 +1057,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{D1EE69C8-A79B-43B1-BCD7-1FC2E49D4961}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{26E5CC9D-E19F-4F94-B73C-628DCC97C5E3}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1152,7 +1067,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{2CD794B7-9E00-4BF1-A36D-8DC6A53AC72F}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{B6ACB932-9C2F-4717-AEEA-3FE086744397}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1165,7 +1080,7 @@
           <xm:sqref>E13:E26 E27:E30 E23:E25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{59585630-447F-4268-A61E-CEAD4CE9232C}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{F48093F0-3980-4DA9-B25C-E7B2C2407088}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1175,7 +1090,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{F5B07463-2461-44F0-AD97-23A1B9E99085}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{1FEB4AB2-267B-40F6-9D59-58AE128B5966}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1185,7 +1100,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{E7FCF23F-2F50-4F9C-B61E-8F9E2873AD3A}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{3392C1E6-6345-4984-899E-4FC140B087DC}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1198,7 +1113,7 @@
           <xm:sqref>F13:F26 F27:F30 F23:F25</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{98F51D84-E84A-4EA5-ABB8-C9E05FC74B86}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{FE87F9CF-634E-4315-B7C0-77D9D15D4766}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1208,7 +1123,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{83DEA64E-7A2E-4FB1-967C-E06894D00029}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{F479DDB3-A8D2-4080-B14D-39F48962F814}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1218,7 +1133,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{AD75D775-6814-40D0-9E12-16962EF02AF3}">
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{BCFB3067-33A6-4830-B640-90752514F21F}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1231,7 +1146,7 @@
           <xm:sqref>E5:E7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{B46C4B29-841B-424A-8A11-C55AB735D129}">
+          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{C08CD84D-13EF-4EEB-8D31-96DF70494340}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1241,7 +1156,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{E06739D0-E548-498E-9577-C938EDF44C57}">
+          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{71CB8D77-C6DE-4693-8D5D-398C98FD5B73}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1251,7 +1166,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{65E5D365-29D2-49E4-A57E-C81222558D43}">
+          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{C0C1C287-BACD-454A-B541-15A249C9EF5A}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1282,7 +1197,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1290,7 +1205,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1298,13 +1213,13 @@
         <v>7</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="31"/>
       <c r="C7" s="29" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1319,7 +1234,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{F939A858-FB70-4FE0-B450-A5A9E78EB11E}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{50BDE54E-AA89-4121-81B3-5240ADE4E4D9}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1329,7 +1244,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{C1A7CA89-6E7B-4F1D-B15F-B01BDA4C7855}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{866B5D2B-3A20-4DA7-BACD-8083DD1CD29F}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1339,7 +1254,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{ABE6E35F-20D2-4C6B-90B5-30EC6E16C2A9}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{513282EB-546D-4364-A6FA-84C77A75A548}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>

</xml_diff>

<commit_message>
Ajout de la fonction de checking de doublon. Ajout total de la mise en forme du excel
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -169,7 +169,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="17">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -271,13 +271,6 @@
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
       <top style="medium"/>
       <bottom style="medium"/>
       <diagonal/>
@@ -322,7 +315,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -423,11 +416,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -443,7 +432,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -912,128 +901,128 @@
       <c r="H13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="19"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="23"/>
+      <c r="B14" s="0"/>
+      <c r="C14" s="0"/>
+      <c r="D14" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="19"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="23"/>
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+      <c r="D15" s="0"/>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="19"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="23"/>
+      <c r="B16" s="0"/>
+      <c r="C16" s="0"/>
+      <c r="D16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="19"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="23"/>
+      <c r="B17" s="0"/>
+      <c r="C17" s="0"/>
+      <c r="D17" s="0"/>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
       <c r="H17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="19"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="23"/>
+      <c r="B18" s="0"/>
+      <c r="C18" s="0"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
       <c r="H18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="19"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="23"/>
+      <c r="B19" s="0"/>
+      <c r="C19" s="0"/>
+      <c r="D19" s="0"/>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="19"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="23"/>
+      <c r="B20" s="0"/>
+      <c r="C20" s="0"/>
+      <c r="D20" s="0"/>
+      <c r="E20" s="0"/>
+      <c r="F20" s="0"/>
+      <c r="G20" s="0"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="19"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="23"/>
+      <c r="B21" s="0"/>
+      <c r="C21" s="0"/>
+      <c r="D21" s="0"/>
+      <c r="E21" s="0"/>
+      <c r="F21" s="0"/>
+      <c r="G21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="19"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="23"/>
+      <c r="B22" s="0"/>
+      <c r="C22" s="0"/>
+      <c r="D22" s="0"/>
+      <c r="E22" s="0"/>
+      <c r="F22" s="0"/>
+      <c r="G22" s="0"/>
       <c r="H22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="19"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="23"/>
+      <c r="B23" s="0"/>
+      <c r="C23" s="0"/>
+      <c r="D23" s="0"/>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0"/>
+      <c r="G23" s="0"/>
       <c r="H23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="19"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="23"/>
+      <c r="B24" s="0"/>
+      <c r="C24" s="0"/>
+      <c r="D24" s="0"/>
+      <c r="E24" s="0"/>
+      <c r="F24" s="0"/>
+      <c r="G24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="19"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="23"/>
+      <c r="B25" s="0"/>
+      <c r="C25" s="0"/>
+      <c r="D25" s="0"/>
+      <c r="E25" s="0"/>
+      <c r="F25" s="0"/>
+      <c r="G25" s="0"/>
       <c r="H25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="19"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="23"/>
+      <c r="B26" s="0"/>
+      <c r="C26" s="0"/>
+      <c r="D26" s="0"/>
+      <c r="E26" s="0"/>
+      <c r="F26" s="0"/>
+      <c r="G26" s="0"/>
       <c r="H26" s="24"/>
     </row>
     <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D27" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>17</v>
-      </c>
+      <c r="D27" s="0"/>
+      <c r="E27" s="0"/>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E39" s="27"/>
+      <c r="E39" s="26"/>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E51" s="27"/>
+      <c r="E51" s="26"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1047,7 +1036,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{B0658272-EA1E-46B9-B6CA-45705880BE4A}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{C2416619-562B-497C-8B41-8DF085AB64C9}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1057,7 +1046,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{26E5CC9D-E19F-4F94-B73C-628DCC97C5E3}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{6A9AD114-EF7E-49F9-BB37-D5975869EE6A}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1067,7 +1056,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{B6ACB932-9C2F-4717-AEEA-3FE086744397}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{522CF061-516A-47B4-9280-B800C6BB8EA2}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1077,10 +1066,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E13:E26 E27:E30 E23:E25</xm:sqref>
+          <xm:sqref>E13:E14 E28:E30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{F48093F0-3980-4DA9-B25C-E7B2C2407088}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{C46BC346-602C-4FD4-8198-BF1F5BDFC28A}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1090,7 +1079,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{1FEB4AB2-267B-40F6-9D59-58AE128B5966}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{BFEE6932-C3B4-4691-9DAA-3E563B638B7C}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1100,7 +1089,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{3392C1E6-6345-4984-899E-4FC140B087DC}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{75A89684-115C-47EA-9250-C34B4F63B4D2}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1110,10 +1099,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>F13:F26 F27:F30 F23:F25</xm:sqref>
+          <xm:sqref>F13 F27:F30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{FE87F9CF-634E-4315-B7C0-77D9D15D4766}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{3F77C090-4AD2-4A40-BB20-58306616E3CE}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1123,7 +1112,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{F479DDB3-A8D2-4080-B14D-39F48962F814}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{B3EAD726-EDDB-4A9C-B0C3-54F6A97968D2}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1133,7 +1122,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{BCFB3067-33A6-4830-B640-90752514F21F}">
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{3EA3FCE0-10A1-422F-9D42-7276E0B0329E}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1146,7 +1135,7 @@
           <xm:sqref>E5:E7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{C08CD84D-13EF-4EEB-8D31-96DF70494340}">
+          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{1092BCD5-37A3-4FA7-9893-759F446FBB4D}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1156,7 +1145,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{71CB8D77-C6DE-4693-8D5D-398C98FD5B73}">
+          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{8EBDC7F4-80BF-4370-9298-E631E3D9F16E}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1166,7 +1155,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{C0C1C287-BACD-454A-B541-15A249C9EF5A}">
+          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{6E66E9C4-835B-4C89-B15E-7EF0584F3E6B}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1176,7 +1165,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E13:E15</xm:sqref>
+          <xm:sqref>E13</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -1193,32 +1182,32 @@
   <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="28" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="28" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="28" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="31"/>
-      <c r="C7" s="29" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="28" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1234,7 +1223,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{50BDE54E-AA89-4121-81B3-5240ADE4E4D9}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{FA8CB6ED-CDFD-4E4C-AA7A-F4EBBA8B88C3}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1244,7 +1233,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{866B5D2B-3A20-4DA7-BACD-8083DD1CD29F}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{B2E5BE3A-1FAA-4C91-9E2B-8D99B5603213}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1254,7 +1243,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{513282EB-546D-4364-A6FA-84C77A75A548}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{B054E0C9-C42C-497F-8FC4-6255E71A20E3}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>

</xml_diff>

<commit_message>
Ajout de la fonction pour mettre les 1 dans le spreadsheet
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t xml:space="preserve">Matrice NOM DU PROJET</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t xml:space="preserve">Pourquoi avoir choisi ce composant ? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pourquoi avoir avoir choisi ce produit ? </t>
   </si>
   <si>
     <t xml:space="preserve">Conforme</t>
@@ -169,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="16">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -271,13 +268,6 @@
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right style="medium"/>
-      <top style="medium"/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="medium"/>
-      <right/>
       <top style="medium"/>
       <bottom style="medium"/>
       <diagonal/>
@@ -315,7 +305,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -416,10 +406,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -432,7 +418,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -901,128 +887,33 @@
       <c r="H13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0"/>
-      <c r="C14" s="0"/>
-      <c r="D14" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-      <c r="D16" s="0"/>
-      <c r="E16" s="0"/>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
+      <c r="D14" s="0"/>
+      <c r="E14" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-      <c r="D17" s="0"/>
-      <c r="E17" s="0"/>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
       <c r="H17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
       <c r="H18" s="24"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
-      <c r="C19" s="0"/>
-      <c r="D19" s="0"/>
-      <c r="E19" s="0"/>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="0"/>
-      <c r="C20" s="0"/>
-      <c r="D20" s="0"/>
-      <c r="E20" s="0"/>
-      <c r="F20" s="0"/>
-      <c r="G20" s="0"/>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="0"/>
-      <c r="C21" s="0"/>
-      <c r="D21" s="0"/>
-      <c r="E21" s="0"/>
-      <c r="F21" s="0"/>
-      <c r="G21" s="0"/>
-    </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="0"/>
-      <c r="C22" s="0"/>
-      <c r="D22" s="0"/>
-      <c r="E22" s="0"/>
-      <c r="F22" s="0"/>
-      <c r="G22" s="0"/>
       <c r="H22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="0"/>
-      <c r="C23" s="0"/>
-      <c r="D23" s="0"/>
-      <c r="E23" s="0"/>
-      <c r="F23" s="0"/>
-      <c r="G23" s="0"/>
       <c r="H23" s="24"/>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="0"/>
-      <c r="C24" s="0"/>
-      <c r="D24" s="0"/>
-      <c r="E24" s="0"/>
-      <c r="F24" s="0"/>
-      <c r="G24" s="0"/>
-    </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="0"/>
-      <c r="C25" s="0"/>
-      <c r="D25" s="0"/>
-      <c r="E25" s="0"/>
-      <c r="F25" s="0"/>
-      <c r="G25" s="0"/>
       <c r="H25" s="24"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="0"/>
-      <c r="C26" s="0"/>
-      <c r="D26" s="0"/>
-      <c r="E26" s="0"/>
-      <c r="F26" s="0"/>
-      <c r="G26" s="0"/>
       <c r="H26" s="24"/>
     </row>
-    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D27" s="0"/>
-      <c r="E27" s="0"/>
-    </row>
+    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E39" s="26"/>
+      <c r="E39" s="25"/>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E51" s="26"/>
+      <c r="E51" s="25"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1036,7 +927,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{C2416619-562B-497C-8B41-8DF085AB64C9}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{90FF33C6-98AA-45E7-A6E0-749E9DE24A1E}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1046,7 +937,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{6A9AD114-EF7E-49F9-BB37-D5975869EE6A}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{1E379030-20FC-43E8-A850-164C67FC20AD}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1056,7 +947,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{522CF061-516A-47B4-9280-B800C6BB8EA2}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{DFCB9770-2F30-4740-BFEC-38264265C55C}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1066,10 +957,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>E13:E14 E28:E30</xm:sqref>
+          <xm:sqref>E13 E28:E30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{C46BC346-602C-4FD4-8198-BF1F5BDFC28A}">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{27828B99-7FC3-4991-AFCE-B5ADE42E26F7}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1079,7 +970,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{BFEE6932-C3B4-4691-9DAA-3E563B638B7C}">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{BD2AD065-9F29-4E51-873D-1D378A2A4192}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1089,7 +980,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{75A89684-115C-47EA-9250-C34B4F63B4D2}">
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{D941FD5A-DEEF-4F98-ADC8-7B9DA0BAA838}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1102,7 +993,7 @@
           <xm:sqref>F13 F27:F30</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{3F77C090-4AD2-4A40-BB20-58306616E3CE}">
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{4E803995-9272-47D0-A13F-DB7AC5516961}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1112,7 +1003,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{B3EAD726-EDDB-4A9C-B0C3-54F6A97968D2}">
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{2E4B7648-2742-46F4-8B56-E99EFBD17CD3}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1122,7 +1013,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{3EA3FCE0-10A1-422F-9D42-7276E0B0329E}">
+          <x14:cfRule type="cellIs" priority="10" operator="equal" id="{EFC01498-82CA-45D1-AB8B-B5BB9AFFC15A}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1135,7 +1026,7 @@
           <xm:sqref>E5:E7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{1092BCD5-37A3-4FA7-9893-759F446FBB4D}">
+          <x14:cfRule type="cellIs" priority="11" operator="equal" id="{6856EFE0-F952-447F-B396-CEBAAE8A7F1F}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1145,7 +1036,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{8EBDC7F4-80BF-4370-9298-E631E3D9F16E}">
+          <x14:cfRule type="cellIs" priority="12" operator="equal" id="{671748DB-3FAD-4916-AF2B-124E6839488D}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1155,7 +1046,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{6E66E9C4-835B-4C89-B15E-7EF0584F3E6B}">
+          <x14:cfRule type="cellIs" priority="13" operator="equal" id="{3F1FD61F-98BB-4299-9186-923B1FDA50F3}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1182,33 +1073,33 @@
   <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="29" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="28" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="27" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="29" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="28" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="29"/>
+      <c r="C7" s="27" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="30"/>
-      <c r="C7" s="28" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1223,7 +1114,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{FA8CB6ED-CDFD-4E4C-AA7A-F4EBBA8B88C3}">
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{979F98E9-E49B-433E-8C28-684D47DA8014}">
             <xm:f>"PC"</xm:f>
             <x14:dxf>
               <fill>
@@ -1233,7 +1124,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{B2E5BE3A-1FAA-4C91-9E2B-8D99B5603213}">
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{5BEC2441-4946-4B30-AB5A-199411DE5DF0}">
             <xm:f>"C"</xm:f>
             <x14:dxf>
               <fill>
@@ -1243,7 +1134,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{B054E0C9-C42C-497F-8FC4-6255E71A20E3}">
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{C29C63F4-1C41-4618-A1EB-331870BA11CB}">
             <xm:f>"NC"</xm:f>
             <x14:dxf>
               <fill>

</xml_diff>